<commit_message>
Refresh historical DataCite versus Scout Excel report
</commit_message>
<xml_diff>
--- a/api-discoveries/reports/REACH_DataCite_Historical_2026-10-28_Scout_Comparison.xlsx
+++ b/api-discoveries/reports/REACH_DataCite_Historical_2026-10-28_Scout_Comparison.xlsx
@@ -149,7 +149,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>150</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -159,7 +159,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -179,7 +179,7 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
@@ -199,7 +199,7 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>103</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
@@ -209,7 +209,7 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -220,7 +220,7 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T15:34:47Z</t>
+          <t xml:space="preserve">2026-10-30T02:33:23Z</t>
         </is>
       </c>
     </row>
@@ -12210,12 +12210,13 @@
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">No addition recommended based on current evidence</t>
         </is>
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical DataCite source identifies award-linked data-management plan; 2026-02-12 DOI-specific DataCite Available date in enrichment; no exact REACH DOI/title. Live DOI/API inaccessible; independent plan document, type and linked outputs not confirmed. Hold without staging.</t>
+          <t xml:space="preserve">Historical DataCite source identifies award-linked data-management plan; 2026-02-12 DOI-specific DataCite Available date in enrichment; no exact REACH DOI/title. Live DOI/API inaccessible; independent plan document, type and linked outputs not confirmed. Hold without staging.
+REACH-SCOUT-2026-10-29-HOURLY-1726ET final bounded recovery: A plan for managing future research data is not the data or research result itself. Close original DOI as NOT_RESEARCH_OUTPUT; independently research eventual outputs.</t>
         </is>
       </c>
       <c r="F3" s="0" t="inlineStr">
@@ -12225,7 +12226,7 @@
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA25OARX459C0174-T1-01</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
@@ -12235,7 +12236,7 @@
       </c>
       <c r="I3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">accessible standalone plan document and public eligibility/type</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J3" s="0" t="inlineStr">
@@ -12260,7 +12261,7 @@
       </c>
       <c r="N3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T00:29:43Z</t>
+          <t xml:space="preserve">2026-10-29T21:30:28.971Z</t>
         </is>
       </c>
     </row>
@@ -12570,12 +12571,13 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTI interview protocol DOI verified by DataCite source and NCAR listing, 2025 Prestley references; parent PRJ-5889 already REACH 000816. Individual component date and scope unresolved.</t>
+          <t xml:space="preserve">HTI interview protocol DOI verified by DataCite source and NCAR listing, 2025 Prestley references; parent PRJ-5889 already REACH 000816. Individual component date and scope unresolved.
+REACH-SCOUT-2026-10-29-HOURLY-1632ET: Second bounded distinct-source round: primary SPARK interview project and NCAR author catalog corroborate the protocol; complete REACH index and exact parent detail confirm PRJ-5889 reach-000816, so component-level duplication remains a genuine human question. Native component date/scope inaccessible.</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
@@ -12585,7 +12587,7 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA21OAR4590206</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
@@ -12595,7 +12597,7 @@
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">record-specific full publication date; public component scope and distinctness</t>
+          <t xml:space="preserve">record-specific full YYYY-MM-DD component publication date; native public interview protocol file scope; separate eligibility versus existing REACH parent reach-000816</t>
         </is>
       </c>
       <c r="J8" s="0" t="inlineStr">
@@ -12620,7 +12622,7 @@
       </c>
       <c r="N8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-28T22:08:00Z</t>
+          <t xml:space="preserve">2026-10-29T20:36:42.360Z</t>
         </is>
       </c>
     </row>
@@ -12786,12 +12788,13 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTI de-identification guide DOI verified by DataCite source and Prestley 2025 reference; parent PRJ-5889 already REACH 000816. Individual component date and scope unresolved.</t>
+          <t xml:space="preserve">HTI de-identification guide DOI verified by DataCite source and Prestley 2025 reference; parent PRJ-5889 already REACH 000816. Individual component date and scope unresolved.
+REACH-SCOUT-2026-10-29-HOURLY-1726ET final bounded recovery: Distinct public guide and full release date unresolved; existing parent may duplicate component. One bounded different-source recovery complete; human review needed, NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F11" s="0" t="inlineStr">
@@ -12801,7 +12804,7 @@
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA21OAR4590206</t>
         </is>
       </c>
       <c r="H11" s="0" t="inlineStr">
@@ -12811,7 +12814,7 @@
       </c>
       <c r="I11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">record-specific full publication date; public component scope and distinctness</t>
+          <t xml:space="preserve">record-specific full YYYY-MM-DD publication date; native public guide/file scope; separate catalog eligibility versus REACH parent reach-000816</t>
         </is>
       </c>
       <c r="J11" s="0" t="inlineStr">
@@ -12836,7 +12839,7 @@
       </c>
       <c r="N11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-28T22:08:00Z</t>
+          <t xml:space="preserve">2026-10-29T21:30:28.971Z</t>
         </is>
       </c>
     </row>
@@ -12858,12 +12861,13 @@
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Minding the Gap broadcast meteorologist/emergency manager survey instrument; historical DataCite lists two NOAA awards, absent exact REACH DOI. NOAA IR 2022 partner survey paper and NWS presentation support workstream, but exact dataset date and public scope unavailable. Hold.</t>
+          <t xml:space="preserve">Minding the Gap broadcast meteorologist/emergency manager survey instrument; historical DataCite lists two NOAA awards, absent exact REACH DOI. NOAA IR 2022 partner survey paper and NWS presentation support workstream, but exact dataset date and public scope unavailable. Hold.
+REACH-SCOUT-2026-10-29-HOURLY-1726ET final bounded recovery: Original survey materials have specific project bridge; native full date and public instrument scope remain unverified. Research complete; human intake pending, NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F12" s="0" t="inlineStr">
@@ -12873,7 +12877,7 @@
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA19OAR0220121, NA19OAR0220192</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
@@ -12883,7 +12887,7 @@
       </c>
       <c r="I12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">record-specific full publication date; public survey instrument scope</t>
+          <t xml:space="preserve">record-specific full YYYY-MM-DD publication date; native public survey instrument/file scope</t>
         </is>
       </c>
       <c r="J12" s="0" t="inlineStr">
@@ -12908,7 +12912,7 @@
       </c>
       <c r="N12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T00:29:43Z</t>
+          <t xml:space="preserve">2026-10-29T21:30:28.971Z</t>
         </is>
       </c>
     </row>
@@ -13002,12 +13006,13 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">DesignSafe experimental dataset DOI linked by ASCE 2022 article; grant NA18OAR4590306 supported. Dataset's exact full publication date unverified; author CV says 2021 only. Metadata blocker seven-day retry; separate 2022 article forwarded as expansion.</t>
+          <t xml:space="preserve">DesignSafe experimental dataset DOI linked by ASCE 2022 article; grant NA18OAR4590306 supported. Dataset's exact full publication date unverified; author CV says 2021 only. Metadata blocker seven-day retry; separate 2022 article forwarded as expansion.
+REACH-SCOUT-2026-10-29-HOURLY-1632ET: Second bounded distinct-source round: SPARK primary project, University of Florida dissertation and author manuscript confirm the dataset's identity and award-specific research; author cites 2021 only, no reliable full date. Linked 2022 article remains a separate already-staged API-seeded expansion; no new batch.</t>
         </is>
       </c>
       <c r="F14" s="0" t="inlineStr">
@@ -13017,7 +13022,7 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA18OAR4590306</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
@@ -13027,7 +13032,7 @@
       </c>
       <c r="I14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">record-specific full YYYY-MM-DD dataset publication date</t>
+          <t xml:space="preserve">record-specific full YYYY-MM-DD DesignSafe dataset publication date; native public file/version validation</t>
         </is>
       </c>
       <c r="J14" s="0" t="inlineStr">
@@ -13052,7 +13057,7 @@
       </c>
       <c r="N14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-28T22:08:00Z</t>
+          <t xml:space="preserve">2026-10-29T20:36:42.360Z</t>
         </is>
       </c>
     </row>
@@ -13434,12 +13439,13 @@
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hurricane Irma tweet documentation dataset; historical DataCite source names NA19OAR0220119, absent exact REACH DOI. Publisher 2023 WCAS paper directly cites this DOI and explicitly acknowledges the same grant; linked article independently verified new and published for human review. Seed dataset release date and parent scope not verified; hold seed only.</t>
+          <t xml:space="preserve">Hurricane Irma tweet documentation dataset; historical DataCite source names NA19OAR0220119, absent exact REACH DOI. Publisher 2023 WCAS paper directly cites this DOI and explicitly acknowledges the same grant; linked article independently verified new and published for human review. Seed dataset release date and parent scope not verified; hold seed only.
+REACH-SCOUT-2026-10-29-HOURLY-1632ET: Second bounded distinct-source round: SPARK primary project and independent author/NCAR dataset listings corroborate identity, but NCAR lists 2025 whereas the cited 2023 Hurricane Irma version 1 may be a component/version. Native DOI inaccessible. The separate 2023 WCAS paper remains previously staged; no duplicate candidate.</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
@@ -13449,7 +13455,7 @@
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA19OAR0220119</t>
         </is>
       </c>
       <c r="H20" s="0" t="inlineStr">
@@ -13459,7 +13465,7 @@
       </c>
       <c r="I20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">record-specific full dataset publication date; public parent project scope</t>
+          <t xml:space="preserve">native full YYYY-MM-DD dataset publication date; version-specific 2023 versus 2025 citation difference; public parent project scope</t>
         </is>
       </c>
       <c r="J20" s="0" t="inlineStr">
@@ -13484,7 +13490,7 @@
       </c>
       <c r="N20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T00:29:43Z</t>
+          <t xml:space="preserve">2026-10-29T20:36:42.360Z</t>
         </is>
       </c>
     </row>
@@ -13722,12 +13728,13 @@
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Minding the Gap interview instruments/analysis methods; DataCite lists two NOAA awards, no exact REACH match. Raw interview data explicitly restricted in source description. NOAA IR survey publication and NWS presentation corroborate workstream, not release date; hold public component until verified.</t>
+          <t xml:space="preserve">Minding the Gap interview instruments/analysis methods; DataCite lists two NOAA awards, no exact REACH match. Raw interview data explicitly restricted in source description. NOAA IR survey publication and NWS presentation corroborate workstream, not release date; hold public component until verified.
+REACH-SCOUT-2026-10-29-HOURLY-1726ET final bounded recovery: Public methods/protocol eligibility and full date unverified; restricted interview responses must not be published. Research complete; human intake pending, NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
@@ -13737,7 +13744,7 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA19OAR0220121, NA19OAR0220192</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
@@ -13747,7 +13754,7 @@
       </c>
       <c r="I24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">record-specific full publication date; public protocol components distinct from restricted raw interview data</t>
+          <t xml:space="preserve">record-specific full YYYY-MM-DD publication date; verified public protocol/method files distinct from restricted participant interview data</t>
         </is>
       </c>
       <c r="J24" s="0" t="inlineStr">
@@ -13772,7 +13779,7 @@
       </c>
       <c r="N24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T00:29:43Z</t>
+          <t xml:space="preserve">2026-10-29T21:30:28.971Z</t>
         </is>
       </c>
     </row>
@@ -14010,12 +14017,13 @@
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-28-HOURLY-2331ET: Original output absent from REACH index; credible seed but unresolved record-specific full publication date; public accessibility and distinctness of HTI interview stimuli files. Hold without staging.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-28-HOURLY-2331ET: Original output absent from REACH index; credible seed but unresolved record-specific full publication date; public accessibility and distinctness of HTI interview stimuli files. Hold without staging.
+REACH-SCOUT-2026-10-29-HOURLY-1726ET final bounded recovery: Full component release date and distinct public scope unresolved; parent version overlap possible. Research complete; human intake pending, NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
@@ -14025,7 +14033,7 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA21OAR4590206</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
@@ -14035,7 +14043,7 @@
       </c>
       <c r="I28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">record-specific full publication date; public accessibility and distinctness of HTI interview stimuli files</t>
+          <t xml:space="preserve">record-specific full YYYY-MM-DD publication date; public accessibility of the stimuli component; distinctness from existing REACH parent reach-000816</t>
         </is>
       </c>
       <c r="J28" s="0" t="inlineStr">
@@ -14060,7 +14068,7 @@
       </c>
       <c r="N28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T03:34:15Z</t>
+          <t xml:space="preserve">2026-10-29T21:30:28.971Z</t>
         </is>
       </c>
     </row>
@@ -14082,12 +14090,13 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-0132ET: DesignSafe Harvey tweet documentation dataset linked to SPARK award NA19OAR0220119; DOI landing and native record full YYYY-MM-DD publication date/public component not retrievable. Related 2024 Morss et al. article DOI 10.1061/nhrefo.nheng-1802 already REACH reach-000789; original dataset independently unresolved. All ten REACH index shards, thirteen prior Scout batches, six SPARK index and six award shards searched for DOI and project match; no exact REACH/Scout DOI. Private human-review status not independently verified.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-0132ET: DesignSafe Harvey tweet documentation dataset linked to SPARK award NA19OAR0220119; DOI landing and native record full YYYY-MM-DD publication date/public component not retrievable. Related 2024 Morss et al. article DOI 10.1061/nhrefo.nheng-1802 already REACH reach-000789; original dataset independently unresolved. All ten REACH index shards, thirteen prior Scout batches, six SPARK index and six award shards searched for DOI and project match; no exact REACH/Scout DOI. Private human-review status not independently verified.
+REACH-SCOUT-2026-10-29-HOURLY-1835ET: ONE bounded different-source follow-up completed. SPARK spark-000237 verifies primary WPO award NA19OAR0220119. Publisher article data availability confirms DesignSafe coding schemes and 2024 article already in REACH reach-000789. NCAR author catalog identifies related DesignSafe DOI 10.17603/ds2-jfsc-8902; component/version relationship unresolved, article date not dataset date. RESEARCH COMPLETE; pending truthful human intake, NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
@@ -14097,7 +14106,7 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA19OAR0220119</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
@@ -14107,7 +14116,7 @@
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">record-specific full YYYY-MM-DD dataset release date; native public DesignSafe component/file scope; overlap with 10.17603/ds2-jfsc-8902</t>
         </is>
       </c>
       <c r="J29" s="0" t="inlineStr">
@@ -14117,7 +14126,7 @@
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Linked 2024 article already REACH; distinct original dataset requires date/public-scope evidence.</t>
+          <t xml:space="preserve">Linked 2024 article already REACH; distinct original dataset requires date/public-scope evidence. No exact original DOI in 1238-row REACH index or 56 Scout batches; related journal article already REACH reach-000789; related DesignSafe DOI requires version comparison.</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
@@ -14132,7 +14141,7 @@
       </c>
       <c r="N29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T05:32:21Z</t>
+          <t xml:space="preserve">2026-10-29T22:36:54.128Z</t>
         </is>
       </c>
     </row>
@@ -14226,12 +14235,13 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical DataCite captured OSF project describes an IDSS exercise method, national emergency-manager survey instrument and after-action reviews. No exact REACH title/DOI in all 1238 index records or 47 Scout findings. OSF landing returned 403 and DOI resolver/API unavailable; full release date and public component scope not independently established.</t>
+          <t xml:space="preserve">Historical DataCite captured OSF project describes an IDSS exercise method, national emergency-manager survey instrument and after-action reviews. No exact REACH title/DOI in all 1238 index records or 47 Scout findings. OSF landing returned 403 and DOI resolver/API unavailable; full release date and public component scope not independently established.
+REACH-SCOUT-2026-10-29-HOURLY-1835ET: ONE bounded different-source follow-up completed. SPARK spark-000248 and official WPO award list independently corroborate primary award NA21OAR4590210 and exact IDSS survey/exercise project. Captured DataCite describes survey instrument, exercise and after-action files, not grant-only notice; native OSF API inaccessible, public file scope and release date unverified. RESEARCH COMPLETE; pending truthful human intake, NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
@@ -14241,7 +14251,7 @@
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA21OAR4590210</t>
         </is>
       </c>
       <c r="H31" s="0" t="inlineStr">
@@ -14251,7 +14261,7 @@
       </c>
       <c r="I31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">public OSF file identities and accessible scope; record-specific full publication date</t>
+          <t xml:space="preserve">native public OSF file identities and accessible component scope; record-specific full YYYY-MM-DD publication date; whether project DOI or individual components merit separate REACH records</t>
         </is>
       </c>
       <c r="J31" s="0" t="inlineStr">
@@ -14261,7 +14271,7 @@
       </c>
       <c r="K31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compared existing REACH records and searched public OSF/project references; no distinct linked publication or code repository with verified output-specific funding confirmed.</t>
+          <t xml:space="preserve">Compared existing REACH records and searched public OSF/project references; no distinct linked publication or code repository with verified output-specific funding confirmed. No exact DOI in complete 1238-row REACH index or 56 Scout candidates; no separately verified expansion output.</t>
         </is>
       </c>
       <c r="L31" s="0" t="inlineStr">
@@ -14276,7 +14286,7 @@
       </c>
       <c r="N31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T01:32:07Z</t>
+          <t xml:space="preserve">2026-10-29T22:36:54.128Z</t>
         </is>
       </c>
     </row>
@@ -14298,12 +14308,13 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical DataCite captured BVOT method-development project. No exact OSF DOI in REACH or staged Scout batches; related BVOT StoryMap and journal works already in REACH reach-000862 and reach-000892. OSF and DOI landing inaccessible; exact date, public files and distinctness unverified.</t>
+          <t xml:space="preserve">Historical DataCite captured BVOT method-development project. No exact OSF DOI in REACH or staged Scout batches; related BVOT StoryMap and journal works already in REACH reach-000862 and reach-000892. OSF and DOI landing inaccessible; exact date, public files and distinctness unverified.
+REACH-SCOUT-2026-10-29-HOURLY-1835ET: ONE bounded different-source follow-up completed. SPARK spark-000249 and official WPO award list verify primary NA21OAR4590212; project-author BVOT tutorial explicitly cites same award. NOAA IR methods article already REACH reach-000892, and REACH contains other BVOT materials. OSF API inaccessible; exact component/version distinction and release date unresolved. RESEARCH COMPLETE; pending truthful human intake, NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
@@ -14313,7 +14324,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA21OAR4590212</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
@@ -14323,7 +14334,7 @@
       </c>
       <c r="I32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">distinctness from existing REACH BVOT outputs; public accessible artifact and full publication date</t>
+          <t xml:space="preserve">native OSF public file identities and release date; distinctness from REACH BVOT StoryMap and journal outputs; separate project DOI eligibility</t>
         </is>
       </c>
       <c r="J32" s="0" t="inlineStr">
@@ -14333,7 +14344,7 @@
       </c>
       <c r="K32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compared existing BVOT StoryMap reach-000862 and publication reach-000892, plus other related BVOT outputs; separate OSF files or version relationships not verified.</t>
+          <t xml:space="preserve">Compared existing BVOT StoryMap reach-000862 and publication reach-000892, plus other related BVOT outputs; separate OSF files or version relationships not verified. REACH BVOT reach-000862, reach-000892, reach-000893, reach-000894 compared; no exact OSF DOI; StoryMap possible expansion requires separate dedup.</t>
         </is>
       </c>
       <c r="L32" s="0" t="inlineStr">
@@ -14348,7 +14359,7 @@
       </c>
       <c r="N32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T01:32:07Z</t>
+          <t xml:space="preserve">2026-10-29T22:36:54.128Z</t>
         </is>
       </c>
     </row>
@@ -14874,12 +14885,13 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">No addition recommended based on current evidence</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Official NOAA IR record confirms distinct 2026 GSL-79 technical memorandum and PDF explicitly acknowledges NOAA cooperative agreement NA19OAR4320073. Complete REACH index and all 47 Scout staged findings have no exact title/DOI. Exact full publication date (YYYY-MM-DD) remains unverified; not forwarded or assigned an invented date.</t>
+          <t xml:space="preserve">Official NOAA IR record confirms distinct 2026 GSL-79 technical memorandum and PDF explicitly acknowledges NOAA cooperative agreement NA19OAR4320073. Complete REACH index and all 47 Scout staged findings have no exact title/DOI. Exact full publication date (YYYY-MM-DD) remains unverified; not forwarded or assigned an invented date.
+REACH-SCOUT-2026-10-29-HOURLY-1632ET: Second bounded project-bridge round: NOAA IR GSL-79 is a genuine report, but five additional official/publisher checks tie it to NOAA Fire Weather Testbed/NGFS and CIRA broad agreement, while SPARK's only match is a different tropical-cyclone MET-TC project. No specific WPO funded deliverable link; no-action, not a metadata-only human referral.</t>
         </is>
       </c>
       <c r="F40" s="0" t="inlineStr">
@@ -14889,7 +14901,7 @@
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA19OAR4320073</t>
         </is>
       </c>
       <c r="H40" s="0" t="inlineStr">
@@ -14909,7 +14921,7 @@
       </c>
       <c r="K40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Examined NOAA Fire Weather Testbed report on NGFS, its 2025 evaluation and its references to NESDIS fire detection and predictive services; no distinct related output with verified NOAA funding and REACH absence confirmed.</t>
+          <t xml:space="preserve">Examined NOAA Fire Weather Testbed report on NGFS, its 2025 evaluation and its references to NESDIS fire detection and predictive services; no distinct related output with verified NOAA funding and REACH absence confirmed. Separate NOAA GSL-71 FWT report DOI 10.25923/4pqf-7g49 and 2025 BAMS Fire Weather Testbed article DOI 10.1175/BAMS-D-24-0204.1 identified; no specific WPO bridge, neither staged.</t>
         </is>
       </c>
       <c r="L40" s="0" t="inlineStr">
@@ -14924,7 +14936,7 @@
       </c>
       <c r="N40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T01:32:07Z</t>
+          <t xml:space="preserve">2026-10-29T20:36:42.360Z</t>
         </is>
       </c>
     </row>
@@ -14946,12 +14958,13 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">No addition recommended based on current evidence</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-28-HOURLY-2331ET: Original output absent from REACH index; credible seed but unresolved record-specific YYYY-MM-DD report publication date; award-to-WPO project scope (broad CIWRO cooperative agreement). Hold without staging.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-28-HOURLY-2331ET: Original output absent from REACH index; credible seed but unresolved record-specific YYYY-MM-DD report publication date; award-to-WPO project scope (broad CIWRO cooperative agreement). Hold without staging.
+REACH-SCOUT-2026-10-29-HOURLY-2026ET: bounded final project-bridge search using NOAA IR, CIWRO/NSSL author/project evidence and all six SPARK award shards. NOAA IR classifies this as an HWT-wide Program &amp; Policy Document with CIWRO base award NA21OAR4320204. Six SPARK award shards reveal only related umbrella use for separate WPO projects, not this FY2025 HWT summary. No project-specific bridge or exact publication day; not eligible for WPO attribution without new positive evidence. Original DOI is a real artifact; no WPO project attribution inferred. No new Hub candidate or private decision.</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
@@ -14961,7 +14974,7 @@
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA21OAR4320204</t>
         </is>
       </c>
       <c r="H41" s="0" t="inlineStr">
@@ -14981,7 +14994,7 @@
       </c>
       <c r="K41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other HWT technical report DOI 10.25923/fcqx-1009 already in REACH; separate seed identity.</t>
+          <t xml:space="preserve">Other HWT technical report DOI 10.25923/fcqx-1009 already in REACH; separate seed identity. Follow-up expansion lead (not verified or staged): HWT FY2025 experiment-specific outputs may be separately researched.</t>
         </is>
       </c>
       <c r="L41" s="0" t="inlineStr">
@@ -14996,7 +15009,7 @@
       </c>
       <c r="N41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T03:34:15Z</t>
+          <t xml:space="preserve">2026-10-30T00:28:49.296091Z</t>
         </is>
       </c>
     </row>
@@ -15306,12 +15319,13 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">No addition recommended based on current evidence</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-0029ET: Original NOAA IR report 'Tornado Tales: 2025 Survey Reference Report' is public and distinct, has DOI and funding field NA21OAR4320204, and is absent from complete 1,238-record REACH index and 12 prior Scout batches. NOAA IR lists year but not exact full YYYY-MM-DD; SPARK award NA21OAR4320204 is shared by several projects and no direct project-specific attribution for this report was confirmed. Do not infer project from broad award or stage without required date.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-0029ET: Original NOAA IR report 'Tornado Tales: 2025 Survey Reference Report' is public and distinct, has DOI and funding field NA21OAR4320204, and is absent from complete 1,238-record REACH index and 12 prior Scout batches. NOAA IR lists year but not exact full YYYY-MM-DD; SPARK award NA21OAR4320204 is shared by several projects and no direct project-specific attribution for this report was confirmed. Do not infer project from broad award or stage without required date.
+REACH-SCOUT-2026-10-29-HOURLY-2026ET: bounded final project-bridge search using NOAA IR, CIWRO/NSSL author/project evidence and all six SPARK award shards. NOAA IR verifies a 2025 Tornado Tales report and CIWRO base award; NSSL/NOAA seminar describes independent NSSL citizen-science survey. Six SPARK award shards show the CIWRO award only as related umbrella for other WPO survey projects. No report-specific WPO funded project bridge or exact YYYY-MM-DD. Original DOI is a real artifact; no WPO project attribution inferred. No new Hub candidate or private decision.</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
@@ -15321,7 +15335,7 @@
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA21OAR4320204</t>
         </is>
       </c>
       <c r="H46" s="0" t="inlineStr">
@@ -15341,7 +15355,7 @@
       </c>
       <c r="K46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Searched related report/topic and WPO project context; no distinct additional verified output staged from this seed in this round.</t>
+          <t xml:space="preserve">Searched related report/topic and WPO project context; no distinct additional verified output staged from this seed in this round. Follow-up expansion lead (not verified or staged): Year-specific Tornado Tales survey reports are distinct NSSL products; no WPO project attribution established.</t>
         </is>
       </c>
       <c r="L46" s="0" t="inlineStr">
@@ -15356,7 +15370,7 @@
       </c>
       <c r="N46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T04:28:11Z</t>
+          <t xml:space="preserve">2026-10-30T00:28:49.296091Z</t>
         </is>
       </c>
     </row>
@@ -15450,12 +15464,13 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">No addition recommended based on current evidence</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-0029ET: Original NOAA IR report 'Developing and Evaluating First-Guess Watch Guidance Within SPC Operations' is public and distinct, has DOI and funding field NA21OAR4320204, and is absent from complete 1,238-record REACH index and 12 prior Scout batches. NOAA IR lists year but not exact full YYYY-MM-DD; SPARK award NA21OAR4320204 is shared by several projects and no direct project-specific attribution for this report was confirmed. Do not infer project from broad award or stage without required date.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-0029ET: Original NOAA IR report 'Developing and Evaluating First-Guess Watch Guidance Within SPC Operations' is public and distinct, has DOI and funding field NA21OAR4320204, and is absent from complete 1,238-record REACH index and 12 prior Scout batches. NOAA IR lists year but not exact full YYYY-MM-DD; SPARK award NA21OAR4320204 is shared by several projects and no direct project-specific attribution for this report was confirmed. Do not infer project from broad award or stage without required date.
+REACH-SCOUT-2026-10-29-HOURLY-2026ET: bounded final project-bridge search using NOAA IR, CIWRO/NSSL author/project evidence and all six SPARK award shards. NOAA IR and independent CIWRO author profile/SPC publication index confirm a 2024 SPC conference paper, but only broad CIWRO base grant NA21OAR4320204 is evidenced. No named WPO-funded SPARK project for this specific SPC guidance work; no exact YYYY-MM-DD. Original DOI is a real artifact; no WPO project attribution inferred. No new Hub candidate or private decision.</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
@@ -15465,7 +15480,7 @@
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA21OAR4320204</t>
         </is>
       </c>
       <c r="H48" s="0" t="inlineStr">
@@ -15485,7 +15500,7 @@
       </c>
       <c r="K48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Searched related report/topic and WPO project context; no distinct additional verified output staged from this seed in this round.</t>
+          <t xml:space="preserve">Searched related report/topic and WPO project context; no distinct additional verified output staged from this seed in this round. Follow-up expansion lead (not verified or staged): Separate 2022 first-guess watch guidance work DOI 10.25923/fssj-fe85 merits project-specific funding check before any candidate.</t>
         </is>
       </c>
       <c r="L48" s="0" t="inlineStr">
@@ -15500,7 +15515,7 @@
       </c>
       <c r="N48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T04:28:11Z</t>
+          <t xml:space="preserve">2026-10-30T00:28:49.296091Z</t>
         </is>
       </c>
     </row>
@@ -15954,12 +15969,13 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">No addition recommended based on current evidence</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-0132ET: NOAA IR identifies WPO office and CIWRO award NA21OAR4320204 for Tornado Tales survey reference report, but SPARK lists base award as RELATED to survey projects; output-specific WPO bridge and full YYYY-MM-DD publication date unverified. Credible candidate; bounded follow-up, not permanent hold. All ten REACH index shards, thirteen prior Scout batches, six SPARK index and six award shards searched for DOI and project match; no exact REACH/Scout DOI. Private human-review status not independently verified.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-0132ET: NOAA IR identifies WPO office and CIWRO award NA21OAR4320204 for Tornado Tales survey reference report, but SPARK lists base award as RELATED to survey projects; output-specific WPO bridge and full YYYY-MM-DD publication date unverified. Credible candidate; bounded follow-up, not permanent hold. All ten REACH index shards, thirteen prior Scout batches, six SPARK index and six award shards searched for DOI and project match; no exact REACH/Scout DOI. Private human-review status not independently verified.
+REACH-SCOUT-2026-10-29-HOURLY-2026ET: bounded final project-bridge search using NOAA IR, CIWRO/NSSL author/project evidence and all six SPARK award shards. NOAA IR WPO office tag and CIWRO base grant are not evidence of a specific WPO-funded project producing the 2026 Tornado Tales report. NSSL/NOAA seminar identify citizen-science program; SPARK award shards show only umbrella related-award connections, no report-specific project bridge. Full publication day unknown. Original DOI is a real artifact; no WPO project attribution inferred. No new Hub candidate or private decision.</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
@@ -15969,7 +15985,7 @@
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">NA21OAR4320204</t>
         </is>
       </c>
       <c r="H55" s="0" t="inlineStr">
@@ -15989,7 +16005,7 @@
       </c>
       <c r="K55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Potential WPO social-science survey relationship not established; inspect project documentation and native report metadata at follow-up.</t>
+          <t xml:space="preserve">Potential WPO social-science survey relationship not established; inspect project documentation and native report metadata at follow-up. Follow-up expansion lead (not verified or staged): NOAA IR WPO office tag is an attribution clue only; not a verified funded project connection.</t>
         </is>
       </c>
       <c r="L55" s="0" t="inlineStr">
@@ -16004,7 +16020,7 @@
       </c>
       <c r="N55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T05:32:21Z</t>
+          <t xml:space="preserve">2026-10-30T00:28:49.296091Z</t>
         </is>
       </c>
     </row>
@@ -23442,17 +23458,18 @@
       </c>
       <c r="D159" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E159" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590367 and matching project workstream; native Zenodo record could not be independently retrieved to establish full date, files or version identity. Missing: Full dataset publication YYYY-MM-DD, native file accessibility, version relation to 21048460. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590367 and matching project workstream; native Zenodo record could not be independently retrieved to establish full date, files or version identity. Missing: Full dataset publication YYYY-MM-DD, native file accessibility, version relation to 21048460. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.
+REACH-SCOUT-2026-10-29-HOURLY-1929ET: One bounded additional-source research round (four source types) completed. Original dataset DOI independently considered; exact primary WPO award NA21OAR4590367 corroborated, but native Zenodo API inaccessible, publication date/files/version family unresolved. Research complete; human decision required; NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F159" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">No exact DOI/title in complete 1238-row public REACH index and 56 pre-existing Scout staged rows; private reviewer status not verifiable.</t>
         </is>
       </c>
       <c r="G159" s="0" t="inlineStr">
@@ -23467,7 +23484,7 @@
       </c>
       <c r="I159" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full dataset publication YYYY-MM-DD, native file accessibility, version relation to 21048460</t>
+          <t xml:space="preserve">exact first-publication YYYY-MM-DD of this DOI; native publicly accessible file scope and version/concept relation to 10.5281/zenodo.21048460</t>
         </is>
       </c>
       <c r="J159" s="0" t="inlineStr">
@@ -23477,7 +23494,7 @@
       </c>
       <c r="K159" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Related Zenodo version/concept DOI identity not assumed to be a distinct output.</t>
+          <t xml:space="preserve">Distinct article/source checked: Shates 2023 study uses separate Marquette observations and is already REACH reach-000132; confirms award and shared Pettersen author but not original Buffalo SCAMP files. 2024/2025 article candidates are separate research outputs, not versions of original Zenodo DOI.</t>
         </is>
       </c>
       <c r="L159" s="0" t="inlineStr">
@@ -23492,7 +23509,7 @@
       </c>
       <c r="N159" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T14:34:00Z</t>
+          <t xml:space="preserve">2026-10-29T23:32:47.760Z</t>
         </is>
       </c>
     </row>
@@ -23514,17 +23531,18 @@
       </c>
       <c r="D160" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E160" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590367 and matching project workstream; native Zenodo record could not be independently retrieved to establish full date, files or version identity. Missing: Full dataset publication YYYY-MM-DD, native file accessibility, version relation to 21048459. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590367 and matching project workstream; native Zenodo record could not be independently retrieved to establish full date, files or version identity. Missing: Full dataset publication YYYY-MM-DD, native file accessibility, version relation to 21048459. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.
+REACH-SCOUT-2026-10-29-HOURLY-1929ET: One bounded additional-source research round (four source types) completed. Original dataset DOI independently considered; exact primary WPO award NA21OAR4590367 corroborated, but native Zenodo API inaccessible, publication date/files/version family unresolved. Research complete; human decision required; NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F160" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">No exact DOI/title in complete 1238-row public REACH index and 56 pre-existing Scout staged rows; private reviewer status not verifiable.</t>
         </is>
       </c>
       <c r="G160" s="0" t="inlineStr">
@@ -23539,7 +23557,7 @@
       </c>
       <c r="I160" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full dataset publication YYYY-MM-DD, native file accessibility, version relation to 21048459</t>
+          <t xml:space="preserve">exact first-publication YYYY-MM-DD of this DOI; native publicly accessible file scope and version/concept relation to 10.5281/zenodo.21048459</t>
         </is>
       </c>
       <c r="J160" s="0" t="inlineStr">
@@ -23549,7 +23567,7 @@
       </c>
       <c r="K160" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Related Zenodo version/concept DOI identity not assumed to be a distinct output.</t>
+          <t xml:space="preserve">Distinct article/source checked: Shates 2023 study uses separate Marquette observations and is already REACH reach-000132; confirms award and shared Pettersen author but not original Buffalo SCAMP files. 2024/2025 article candidates are separate research outputs, not versions of original Zenodo DOI.</t>
         </is>
       </c>
       <c r="L160" s="0" t="inlineStr">
@@ -23564,7 +23582,7 @@
       </c>
       <c r="N160" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T14:34:00Z</t>
+          <t xml:space="preserve">2026-10-29T23:32:47.760Z</t>
         </is>
       </c>
     </row>
@@ -23586,17 +23604,18 @@
       </c>
       <c r="D161" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E161" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA22OAR4590188 and matching project workstream; native Zenodo record could not be independently retrieved to establish full date, files or version identity. Missing: Full source-code publication YYYY-MM-DD, native files, version relation to 23044470. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA22OAR4590188 and matching project workstream; native Zenodo record could not be independently retrieved to establish full date, files or version identity. Missing: Full source-code publication YYYY-MM-DD, native files, version relation to 23044470. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.
+REACH-SCOUT-2026-10-29-HOURLY-1929ET: One bounded additional-source research round (four source types) completed. Original software DOI independently considered; exact primary WPO award NA22OAR4590188 corroborated, but native Zenodo API inaccessible, publication date/files/version family unresolved. Research complete; human decision required; NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F161" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">No exact DOI/title in complete 1238-row public REACH index and 56 pre-existing Scout staged rows; private reviewer status not verifiable.</t>
         </is>
       </c>
       <c r="G161" s="0" t="inlineStr">
@@ -23611,7 +23630,7 @@
       </c>
       <c r="I161" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full source-code publication YYYY-MM-DD, native files, version relation to 23044470</t>
+          <t xml:space="preserve">exact first-publication YYYY-MM-DD of this DOI; native publicly accessible file scope and version/concept relation to 10.5281/zenodo.23044470</t>
         </is>
       </c>
       <c r="J161" s="0" t="inlineStr">
@@ -23621,7 +23640,7 @@
       </c>
       <c r="K161" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Related Zenodo version/concept DOI identity not assumed to be a distinct output.</t>
+          <t xml:space="preserve">Distinct article/source checked: Yeo 2024 paper identifies same WPO JTTI award and shared investigator Fujisaki-Manome; not proof of exact native FVCOM source archive release. 2024/2025 article candidates are separate research outputs, not versions of original Zenodo DOI.</t>
         </is>
       </c>
       <c r="L161" s="0" t="inlineStr">
@@ -23636,7 +23655,7 @@
       </c>
       <c r="N161" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T14:34:00Z</t>
+          <t xml:space="preserve">2026-10-29T23:32:47.760Z</t>
         </is>
       </c>
     </row>
@@ -23658,17 +23677,18 @@
       </c>
       <c r="D162" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E162" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA22OAR4590188 and matching project workstream; native Zenodo record could not be independently retrieved to establish full date, files or version identity. Missing: Full source-code publication YYYY-MM-DD, native files, version relation to 23044469. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA22OAR4590188 and matching project workstream; native Zenodo record could not be independently retrieved to establish full date, files or version identity. Missing: Full source-code publication YYYY-MM-DD, native files, version relation to 23044469. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.
+REACH-SCOUT-2026-10-29-HOURLY-1929ET: One bounded additional-source research round (four source types) completed. Original software DOI independently considered; exact primary WPO award NA22OAR4590188 corroborated, but native Zenodo API inaccessible, publication date/files/version family unresolved. Research complete; human decision required; NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F162" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">No exact DOI/title in complete 1238-row public REACH index and 56 pre-existing Scout staged rows; private reviewer status not verifiable.</t>
         </is>
       </c>
       <c r="G162" s="0" t="inlineStr">
@@ -23683,7 +23703,7 @@
       </c>
       <c r="I162" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full source-code publication YYYY-MM-DD, native files, version relation to 23044469</t>
+          <t xml:space="preserve">exact first-publication YYYY-MM-DD of this DOI; native publicly accessible file scope and version/concept relation to 10.5281/zenodo.23044469</t>
         </is>
       </c>
       <c r="J162" s="0" t="inlineStr">
@@ -23693,7 +23713,7 @@
       </c>
       <c r="K162" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Related Zenodo version/concept DOI identity not assumed to be a distinct output.</t>
+          <t xml:space="preserve">Distinct article/source checked: Yeo 2024 paper identifies same WPO JTTI award and shared investigator Fujisaki-Manome; not proof of exact native FVCOM source archive release. 2024/2025 article candidates are separate research outputs, not versions of original Zenodo DOI.</t>
         </is>
       </c>
       <c r="L162" s="0" t="inlineStr">
@@ -23708,7 +23728,7 @@
       </c>
       <c r="N162" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T14:34:00Z</t>
+          <t xml:space="preserve">2026-10-29T23:32:47.760Z</t>
         </is>
       </c>
     </row>
@@ -23730,17 +23750,18 @@
       </c>
       <c r="D163" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E163" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA22OAR0110487 and matching project workstream; native Zenodo record could not be independently retrieved to establish full date, files or version identity. Missing: Full dataset publication YYYY-MM-DD, native files, version relation to 23289231. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA22OAR0110487 and matching project workstream; native Zenodo record could not be independently retrieved to establish full date, files or version identity. Missing: Full dataset publication YYYY-MM-DD, native files, version relation to 23289231. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.
+REACH-SCOUT-2026-10-29-HOURLY-1929ET: One bounded additional-source research round (four source types) completed. Original dataset DOI independently considered; exact primary WPO award NA22OAR0110487 corroborated, but native Zenodo API inaccessible, publication date/files/version family unresolved. Research complete; human decision required; NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F163" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">No exact DOI/title in complete 1238-row public REACH index and 56 pre-existing Scout staged rows; private reviewer status not verifiable.</t>
         </is>
       </c>
       <c r="G163" s="0" t="inlineStr">
@@ -23755,7 +23776,7 @@
       </c>
       <c r="I163" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full dataset publication YYYY-MM-DD, native files, version relation to 23289231</t>
+          <t xml:space="preserve">exact first-publication YYYY-MM-DD of this DOI; native publicly accessible file scope and version/concept relation to 10.5281/zenodo.23289231</t>
         </is>
       </c>
       <c r="J163" s="0" t="inlineStr">
@@ -23765,7 +23786,7 @@
       </c>
       <c r="K163" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Related Zenodo version/concept DOI identity not assumed to be a distinct output.</t>
+          <t xml:space="preserve">Distinct article/source checked: Xu/Zaron 2025 paper identifies exact WPO grant and MOM6 simulation, but availability points to distinct Zenodo DOI 16905128; original DOI files/date not verified. 2024/2025 article candidates are separate research outputs, not versions of original Zenodo DOI.</t>
         </is>
       </c>
       <c r="L163" s="0" t="inlineStr">
@@ -23780,7 +23801,7 @@
       </c>
       <c r="N163" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T14:34:00Z</t>
+          <t xml:space="preserve">2026-10-29T23:32:47.760Z</t>
         </is>
       </c>
     </row>
@@ -23802,17 +23823,18 @@
       </c>
       <c r="D164" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E164" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA22OAR0110487 and matching project workstream; native Zenodo record could not be independently retrieved to establish full date, files or version identity. Missing: Full dataset publication YYYY-MM-DD, native files, version relation to 23289230. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA22OAR0110487 and matching project workstream; native Zenodo record could not be independently retrieved to establish full date, files or version identity. Missing: Full dataset publication YYYY-MM-DD, native files, version relation to 23289230. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.
+REACH-SCOUT-2026-10-29-HOURLY-1929ET: One bounded additional-source research round (four source types) completed. Original dataset DOI independently considered; exact primary WPO award NA22OAR0110487 corroborated, but native Zenodo API inaccessible, publication date/files/version family unresolved. Research complete; human decision required; NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F164" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">No exact DOI/title in complete 1238-row public REACH index and 56 pre-existing Scout staged rows; private reviewer status not verifiable.</t>
         </is>
       </c>
       <c r="G164" s="0" t="inlineStr">
@@ -23827,7 +23849,7 @@
       </c>
       <c r="I164" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full dataset publication YYYY-MM-DD, native files, version relation to 23289230</t>
+          <t xml:space="preserve">exact first-publication YYYY-MM-DD of this DOI; native publicly accessible file scope and version/concept relation to 10.5281/zenodo.23289230</t>
         </is>
       </c>
       <c r="J164" s="0" t="inlineStr">
@@ -23837,7 +23859,7 @@
       </c>
       <c r="K164" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Related Zenodo version/concept DOI identity not assumed to be a distinct output.</t>
+          <t xml:space="preserve">Distinct article/source checked: Xu/Zaron 2025 paper identifies exact WPO grant and MOM6 simulation, but availability points to distinct Zenodo DOI 16905128; original DOI files/date not verified. 2024/2025 article candidates are separate research outputs, not versions of original Zenodo DOI.</t>
         </is>
       </c>
       <c r="L164" s="0" t="inlineStr">
@@ -23852,7 +23874,7 @@
       </c>
       <c r="N164" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T14:34:00Z</t>
+          <t xml:space="preserve">2026-10-29T23:32:47.760Z</t>
         </is>
       </c>
     </row>
@@ -23946,12 +23968,13 @@
       </c>
       <c r="D166" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Sent to Discovery Hub for review</t>
         </is>
       </c>
       <c r="E166" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590374; Scripps NOPP NHCI official catalog corroborates sensor/first-five family, but does not establish full publication day or all alternate DOI identities. Missing: Exact first-publication YYYY-MM-DD and public ERDDAP data scope. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590374; Scripps NOPP NHCI official catalog corroborates sensor/first-five family, but does not establish full publication day or all alternate DOI identities. Missing: Exact first-publication YYYY-MM-DD and public ERDDAP data scope. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.
+REACH-SCOUT-2026-10-29-HOURLY-1835ET: ONE bounded different-source follow-up completed. SPARK spark-000336 primary NA21OAR4590374. Scripps publisher catalog distinguishes 2022 sensor S93W23 from 2022 first-five S9059K; live ERDDAP resolves exact DOI and public sensor variables, license and observation dates, but not publication date. RESEARCH COMPLETE; pending truthful human intake, NOT DELIVERED TO HUB.\nREACH-SCOUT-2026-10-30-HOURLY-1435ET: Executive DataCite created Pub Date accepted; exact DOI staged in manifest-verified 1229ET four-row normal-review batch; previous automated metadata status preserved in history; private Hub import and reviewer decision NOT VERIFIED.</t>
         </is>
       </c>
       <c r="F166" s="0" t="inlineStr">
@@ -23971,17 +23994,17 @@
       </c>
       <c r="I166" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exact first-publication YYYY-MM-DD and public ERDDAP data scope</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J166" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">https://github.com/PART-WPO/reach-scout-discoveries/blob/main/scout-discoveries/batches/2026-10-30-hourly-1229ET-nhci-date-policy-normal-review-001.csv</t>
         </is>
       </c>
       <c r="K166" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Separate year-specific NHCI sensor/first-five data; S9TG60 versus S9PP42 identity conflict requires native publisher resolution.</t>
+          <t xml:space="preserve">Separate year-specific NHCI sensor/first-five data; S9TG60 versus S9PP42 identity conflict requires native publisher resolution. No exact DOI in 1238-row REACH index or 56 Scout batches; sensor data distinct from first-five data.</t>
         </is>
       </c>
       <c r="L166" s="0" t="inlineStr">
@@ -23996,7 +24019,7 @@
       </c>
       <c r="N166" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T14:34:00Z</t>
+          <t xml:space="preserve">2026-10-29T22:36:54.128Z</t>
         </is>
       </c>
     </row>
@@ -24234,12 +24257,13 @@
       </c>
       <c r="D170" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Sent to Discovery Hub for review</t>
         </is>
       </c>
       <c r="E170" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590374; Scripps NOPP NHCI official catalog corroborates sensor/first-five family, but does not establish full publication day or all alternate DOI identities. Missing: Exact first-publication YYYY-MM-DD and separate first-five vs sensor identity. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590374; Scripps NOPP NHCI official catalog corroborates sensor/first-five family, but does not establish full publication day or all alternate DOI identities. Missing: Exact first-publication YYYY-MM-DD and separate first-five vs sensor identity. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.
+REACH-SCOUT-2026-10-29-HOURLY-1835ET: ONE bounded different-source follow-up completed. SPARK spark-000336 primary NA21OAR4590374. Scripps publisher catalog distinguishes 2024 first-five S9F59M from 2024 sensor S9K013; live ERDDAP resolves exact DOI and public wave coefficient variables, license and observation dates, but not publication date. RESEARCH COMPLETE; pending truthful human intake, NOT DELIVERED TO HUB.\nREACH-SCOUT-2026-10-30-HOURLY-1435ET: Executive DataCite created Pub Date accepted; exact DOI staged in manifest-verified 1229ET four-row normal-review batch; previous automated metadata status preserved in history; private Hub import and reviewer decision NOT VERIFIED.</t>
         </is>
       </c>
       <c r="F170" s="0" t="inlineStr">
@@ -24259,17 +24283,17 @@
       </c>
       <c r="I170" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exact first-publication YYYY-MM-DD and separate first-five vs sensor identity</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J170" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">https://github.com/PART-WPO/reach-scout-discoveries/blob/main/scout-discoveries/batches/2026-10-30-hourly-1229ET-nhci-date-policy-normal-review-001.csv</t>
         </is>
       </c>
       <c r="K170" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Separate year-specific NHCI sensor/first-five data; S9TG60 versus S9PP42 identity conflict requires native publisher resolution.</t>
+          <t xml:space="preserve">Separate year-specific NHCI sensor/first-five data; S9TG60 versus S9PP42 identity conflict requires native publisher resolution. No exact DOI in 1238-row REACH index or 56 Scout batches; first-five data distinct from sensor data.</t>
         </is>
       </c>
       <c r="L170" s="0" t="inlineStr">
@@ -24284,7 +24308,7 @@
       </c>
       <c r="N170" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T14:34:00Z</t>
+          <t xml:space="preserve">2026-10-29T22:36:54.128Z</t>
         </is>
       </c>
     </row>
@@ -24306,12 +24330,13 @@
       </c>
       <c r="D171" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E171" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Pacific DWSD first-five wave data; direct WPO drifter award captured, but exact dataset publication date and public scope not independently verified. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Pacific DWSD first-five wave data; direct WPO drifter award captured, but exact dataset publication date and public scope not independently verified. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.
+REACH-SCOUT-2026-10-29-HOURLY-2229ET: One substantive bounded different-source recovery round; Publisher general data policy and GDP funding examined; exact native dataset date/scope not retrievable. Full REACH index 10/10 and detail 140/140 shards, SPARK 6/6 index, and Scout 17 immutable batches/59 rows checked; no exact original DOI/title match. Missing metadata and version questions require human decision; NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F171" s="0" t="inlineStr">
@@ -24356,7 +24381,7 @@
       </c>
       <c r="N171" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T15:34:47Z</t>
+          <t xml:space="preserve">2026-10-30T02:33:23Z</t>
         </is>
       </c>
     </row>
@@ -24450,12 +24475,13 @@
       </c>
       <c r="D173" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Sent to Discovery Hub for review</t>
         </is>
       </c>
       <c r="E173" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590374; Scripps NOPP NHCI official catalog corroborates sensor/first-five family, but does not establish full publication day or all alternate DOI identities. Missing: Exact first-publication YYYY-MM-DD and public ERDDAP data scope. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590374; Scripps NOPP NHCI official catalog corroborates sensor/first-five family, but does not establish full publication day or all alternate DOI identities. Missing: Exact first-publication YYYY-MM-DD and public ERDDAP data scope. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.
+REACH-SCOUT-2026-10-29-HOURLY-2129ET: distinct-source follow-up: native Scripps ERDDAP confirms original DOI, public data variables and observation period (not publication date); primary SPARK project spark-000336 directly funds drifting buoy observations with award NA21OAR4590374; all 10 public REACH index shards (1,238 rows) and all 17 Scout batches (59 proposals) rechecked with no exact DOI/title match. Full REACH detail and private Hub not verified. Research complete, pending human intake. \nREACH-SCOUT-2026-10-30-HOURLY-1435ET: Executive DataCite created Pub Date accepted; exact DOI staged in manifest-verified 1229ET four-row normal-review batch; previous automated metadata status preserved in history; private Hub import and reviewer decision NOT VERIFIED.</t>
         </is>
       </c>
       <c r="F173" s="0" t="inlineStr">
@@ -24475,12 +24501,12 @@
       </c>
       <c r="I173" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exact first-publication YYYY-MM-DD and public ERDDAP data scope</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J173" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">https://github.com/PART-WPO/reach-scout-discoveries/blob/main/scout-discoveries/batches/2026-10-30-hourly-1229ET-nhci-date-policy-normal-review-001.csv</t>
         </is>
       </c>
       <c r="K173" s="0" t="inlineStr">
@@ -24500,7 +24526,7 @@
       </c>
       <c r="N173" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T14:34:00Z</t>
+          <t xml:space="preserve">2026-10-30T01:29:29.347Z</t>
         </is>
       </c>
     </row>
@@ -24522,12 +24548,13 @@
       </c>
       <c r="D174" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E174" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Pacific DWSD sensor data; direct WPO drifter award captured, but first publication date and distinctness from first-five coefficients unresolved. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Pacific DWSD sensor data; direct WPO drifter award captured, but first publication date and distinctness from first-five coefficients unresolved. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.
+REACH-SCOUT-2026-10-29-HOURLY-2229ET: One substantive bounded different-source recovery round; Publisher general data policy and GDP funding examined; exact native dataset date/scope not retrievable. Full REACH index 10/10 and detail 140/140 shards, SPARK 6/6 index, and Scout 17 immutable batches/59 rows checked; no exact original DOI/title match. Missing metadata and version questions require human decision; NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F174" s="0" t="inlineStr">
@@ -24572,7 +24599,7 @@
       </c>
       <c r="N174" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T15:34:47Z</t>
+          <t xml:space="preserve">2026-10-30T02:33:23Z</t>
         </is>
       </c>
     </row>
@@ -24666,12 +24693,13 @@
       </c>
       <c r="D176" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E176" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590374; Scripps NOPP NHCI official catalog corroborates sensor/first-five family, but does not establish full publication day or all alternate DOI identities. Missing: Exact first-publication YYYY-MM-DD and separate first-five vs sensor identity. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590374; Scripps NOPP NHCI official catalog corroborates sensor/first-five family, but does not establish full publication day or all alternate DOI identities. Missing: Exact first-publication YYYY-MM-DD and separate first-five vs sensor identity. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.
+REACH-SCOUT-2026-10-29-HOURLY-2229ET: One substantive bounded different-source recovery round; Publisher lists S9PP42 but DOI tombstones; S9TG60 shares captured title, and a different 2025 targeted-storm DOI exists. Full REACH index 10/10 and detail 140/140 shards, SPARK 6/6 index, and Scout 17 immutable batches/59 rows checked; no exact original DOI/title match. Missing metadata and version questions require human decision; NOT DELIVERED TO HUB.\nREACH-SCOUT-2026-10-30-HOURLY-1435ET: Reconciled reach_snapshot to verified public REACH manifest SHA and removed date-only missing evidence; canonical DOI/version remains a real human intake question. No private Hub import claimed.</t>
         </is>
       </c>
       <c r="F176" s="0" t="inlineStr">
@@ -24691,7 +24719,7 @@
       </c>
       <c r="I176" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exact first-publication YYYY-MM-DD and separate first-five vs sensor identity</t>
+          <t xml:space="preserve">Resolve canonical 2023 first-five DOI versus alternate S9TG60</t>
         </is>
       </c>
       <c r="J176" s="0" t="inlineStr">
@@ -24716,7 +24744,7 @@
       </c>
       <c r="N176" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T14:34:00Z</t>
+          <t xml:space="preserve">2026-10-30T02:33:23Z</t>
         </is>
       </c>
     </row>
@@ -24738,12 +24766,13 @@
       </c>
       <c r="D177" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E177" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Atlantic 2024 GTS drifter dataset; LDL cites WPO award but its webpage shows DOI S9QP4CD while captured DOI is S9QP4C; confirm identity and publication date. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Atlantic 2024 GTS drifter dataset; LDL cites WPO award but its webpage shows DOI S9QP4CD while captured DOI is S9QP4C; confirm identity and publication date. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.
+REACH-SCOUT-2026-10-29-HOURLY-2129ET: distinct-source follow-up: native Scripps ERDDAP confirms original DOI, public data variables and observation period (not publication date); primary SPARK project spark-000336 directly funds drifting buoy observations with award NA21OAR4590374; all 10 public REACH index shards (1,238 rows) and all 17 Scout batches (59 proposals) rechecked with no exact DOI/title match. Full REACH detail and private Hub not verified. Research complete, pending human intake. Scripps catalog cites S9QP4CD, but native ERDDAP identifies S9QP4C; unresolved publisher typo.</t>
         </is>
       </c>
       <c r="F177" s="0" t="inlineStr">
@@ -24763,7 +24792,7 @@
       </c>
       <c r="I177" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">record-specific first publication date (YYYY-MM-DD); native repository version/identity and public scope confirmation</t>
+          <t xml:space="preserve">record-specific first-publication YYYY-MM-DD; publisher catalog DOI S9QP4CD vs native DOI S9QP4C discrepancy</t>
         </is>
       </c>
       <c r="J177" s="0" t="inlineStr">
@@ -24788,7 +24817,7 @@
       </c>
       <c r="N177" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T15:34:47Z</t>
+          <t xml:space="preserve">2026-10-30T01:29:29.347Z</t>
         </is>
       </c>
     </row>
@@ -24810,12 +24839,13 @@
       </c>
       <c r="D178" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E178" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Atlantic 2022 GTS drifter dataset; LDL identifies WPO award and 2023 citation year, not exact first-publication date. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Atlantic 2022 GTS drifter dataset; LDL identifies WPO award and 2023 citation year, not exact first-publication date. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.
+REACH-SCOUT-2026-10-29-HOURLY-2229ET: One substantive bounded different-source recovery round; Native ERDDAP verifies 2022 observation season and DOI; citation year/observation dates are not release date. Full REACH index 10/10 and detail 140/140 shards, SPARK 6/6 index, and Scout 17 immutable batches/59 rows checked; no exact original DOI/title match. Missing metadata and version questions require human decision; NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F178" s="0" t="inlineStr">
@@ -24860,7 +24890,7 @@
       </c>
       <c r="N178" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T15:34:47Z</t>
+          <t xml:space="preserve">2026-10-30T02:33:23Z</t>
         </is>
       </c>
     </row>
@@ -24882,12 +24912,13 @@
       </c>
       <c r="D179" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E179" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590374; Scripps NOPP NHCI official catalog corroborates sensor/first-five family, but does not establish full publication day or all alternate DOI identities. Missing: Exact first-publication YYYY-MM-DD and whether this is an alternate/version of S9PP42 rather than distinct dataset. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590374; Scripps NOPP NHCI official catalog corroborates sensor/first-five family, but does not establish full publication day or all alternate DOI identities. Missing: Exact first-publication YYYY-MM-DD and whether this is an alternate/version of S9PP42 rather than distinct dataset. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.
+REACH-SCOUT-2026-10-29-HOURLY-2229ET: One substantive bounded different-source recovery round; Publisher lists S9PP42 but DOI tombstones; S9TG60 shares captured title, and a different 2025 targeted-storm DOI exists. Full REACH index 10/10 and detail 140/140 shards, SPARK 6/6 index, and Scout 17 immutable batches/59 rows checked; no exact original DOI/title match. Missing metadata and version questions require human decision; NOT DELIVERED TO HUB.\nREACH-SCOUT-2026-10-30-HOURLY-1435ET: Reconciled reach_snapshot to verified public REACH manifest SHA and removed date-only missing evidence; canonical DOI/version remains a real human intake question. No private Hub import claimed.</t>
         </is>
       </c>
       <c r="F179" s="0" t="inlineStr">
@@ -24907,7 +24938,7 @@
       </c>
       <c r="I179" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exact first-publication YYYY-MM-DD and whether this is an alternate/version of S9PP42 rather than distinct dataset</t>
+          <t xml:space="preserve">Resolve alternate/version relationship to S9PP42 and canonical 2023 first-five DOI</t>
         </is>
       </c>
       <c r="J179" s="0" t="inlineStr">
@@ -24932,7 +24963,7 @@
       </c>
       <c r="N179" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T14:34:00Z</t>
+          <t xml:space="preserve">2026-10-30T02:33:23Z</t>
         </is>
       </c>
     </row>
@@ -24954,12 +24985,13 @@
       </c>
       <c r="D180" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E180" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Atlantic 2023 GTS drifter dataset; LDL identifies WPO award and citation year only; exact date unresolved. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Atlantic 2023 GTS drifter dataset; LDL identifies WPO award and citation year only; exact date unresolved. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.
+REACH-SCOUT-2026-10-29-HOURLY-2229ET: One substantive bounded different-source recovery round; Native ERDDAP verifies 2023 observation season and DOI; citation year/observation dates are not release date. Full REACH index 10/10 and detail 140/140 shards, SPARK 6/6 index, and Scout 17 immutable batches/59 rows checked; no exact original DOI/title match. Missing metadata and version questions require human decision; NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F180" s="0" t="inlineStr">
@@ -25004,7 +25036,7 @@
       </c>
       <c r="N180" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T15:34:47Z</t>
+          <t xml:space="preserve">2026-10-30T02:33:23Z</t>
         </is>
       </c>
     </row>
@@ -25026,12 +25058,13 @@
       </c>
       <c r="D181" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E181" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Atlantic 2021 GTS drifter dataset; LDL identifies WPO award and 2023 citation year, not exact date. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Atlantic 2021 GTS drifter dataset; LDL identifies WPO award and 2023 citation year, not exact date. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.
+REACH-SCOUT-2026-10-29-HOURLY-2229ET: One substantive bounded different-source recovery round; Native ERDDAP verifies 2021 observation season and DOI; citation year/observation dates are not release date. Full REACH index 10/10 and detail 140/140 shards, SPARK 6/6 index, and Scout 17 immutable batches/59 rows checked; no exact original DOI/title match. Missing metadata and version questions require human decision; NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F181" s="0" t="inlineStr">
@@ -25076,7 +25109,7 @@
       </c>
       <c r="N181" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T15:34:47Z</t>
+          <t xml:space="preserve">2026-10-30T02:33:23Z</t>
         </is>
       </c>
     </row>
@@ -25098,12 +25131,13 @@
       </c>
       <c r="D182" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Sent to Discovery Hub for review</t>
         </is>
       </c>
       <c r="E182" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590374; Scripps NOPP NHCI official catalog corroborates sensor/first-five family, but does not establish full publication day or all alternate DOI identities. Missing: Exact first-publication YYYY-MM-DD and public ERDDAP data scope. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1031ET: First bounded round (five distinct source checks). Captured DataCite structured fundingReference identifies exact WPO primary SPARK award NA21OAR4590374; Scripps NOPP NHCI official catalog corroborates sensor/first-five family, but does not establish full publication day or all alternate DOI identities. Missing: Exact first-publication YYYY-MM-DD and public ERDDAP data scope. Retry only on or after 2026-11-05T14:34:00Z using genuinely different authoritative source; then human_metadata_needed or evidenced no-action, no repeated reset.
+REACH-SCOUT-2026-10-29-HOURLY-2129ET: distinct-source follow-up: native Scripps ERDDAP confirms original DOI, public data variables and observation period (not publication date); primary SPARK project spark-000336 directly funds drifting buoy observations with award NA21OAR4590374; all 10 public REACH index shards (1,238 rows) and all 17 Scout batches (59 proposals) rechecked with no exact DOI/title match. Full REACH detail and private Hub not verified. Research complete, pending human intake. \nREACH-SCOUT-2026-10-30-HOURLY-1435ET: Executive DataCite created Pub Date accepted; exact DOI staged in manifest-verified 1229ET four-row normal-review batch; previous automated metadata status preserved in history; private Hub import and reviewer decision NOT VERIFIED.</t>
         </is>
       </c>
       <c r="F182" s="0" t="inlineStr">
@@ -25123,12 +25157,12 @@
       </c>
       <c r="I182" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exact first-publication YYYY-MM-DD and public ERDDAP data scope</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J182" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">https://github.com/PART-WPO/reach-scout-discoveries/blob/main/scout-discoveries/batches/2026-10-30-hourly-1229ET-nhci-date-policy-normal-review-001.csv</t>
         </is>
       </c>
       <c r="K182" s="0" t="inlineStr">
@@ -25148,7 +25182,7 @@
       </c>
       <c r="N182" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T14:34:00Z</t>
+          <t xml:space="preserve">2026-10-30T01:29:29.347Z</t>
         </is>
       </c>
     </row>
@@ -25314,12 +25348,13 @@
       </c>
       <c r="D185" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E185" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: VORTEX-SE polarimetric/lightning poster; direct WPO award and ORCID date 2023-07-12, but native Figshare first-publication date and version identity unverified. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: VORTEX-SE polarimetric/lightning poster; direct WPO award and ORCID date 2023-07-12, but native Figshare first-publication date and version identity unverified. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.
+REACH-SCOUT-2026-10-29-HOURLY-2229ET: One substantive bounded different-source recovery round; AMS 30th SLS confirms exact poster; ORCID Figshare-sourced 2023-07-12; Figshare API inaccessible; concept/v1 are same output family. Full REACH index 10/10 and detail 140/140 shards, SPARK 6/6 index, and Scout 17 immutable batches/59 rows checked; no exact original DOI/title match. Missing metadata and version questions require human decision; NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F185" s="0" t="inlineStr">
@@ -25364,7 +25399,7 @@
       </c>
       <c r="N185" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T15:34:47Z</t>
+          <t xml:space="preserve">2026-10-30T02:33:23Z</t>
         </is>
       </c>
     </row>
@@ -25386,12 +25421,13 @@
       </c>
       <c r="D186" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E186" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Version 1 of same VORTEX-SE poster; verify native Figshare date and relationship to concept DOI, do not double count. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Version 1 of same VORTEX-SE poster; verify native Figshare date and relationship to concept DOI, do not double count. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.
+REACH-SCOUT-2026-10-29-HOURLY-2229ET: One substantive bounded different-source recovery round; AMS 30th SLS confirms exact poster; ORCID Figshare-sourced 2023-07-12; Figshare API inaccessible; concept/v1 are same output family. Full REACH index 10/10 and detail 140/140 shards, SPARK 6/6 index, and Scout 17 immutable batches/59 rows checked; no exact original DOI/title match. Missing metadata and version questions require human decision; NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F186" s="0" t="inlineStr">
@@ -25436,7 +25472,7 @@
       </c>
       <c r="N186" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T15:34:47Z</t>
+          <t xml:space="preserve">2026-10-30T02:33:23Z</t>
         </is>
       </c>
     </row>
@@ -25458,12 +25494,13 @@
       </c>
       <c r="D187" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E187" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: ELDORA ML QC dataset directly linked by funded AMS article; exact Figshare dataset publication date and version identity unverified. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: ELDORA ML QC dataset directly linked by funded AMS article; exact Figshare dataset publication date and version identity unverified. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.
+REACH-SCOUT-2026-10-29-HOURLY-2229ET: One substantive bounded different-source recovery round; AMS article explicitly links exact dataset and WPO award; NOAA IR corroborates; Figshare API inaccessible; concept/v1 are same output family. Full REACH index 10/10 and detail 140/140 shards, SPARK 6/6 index, and Scout 17 immutable batches/59 rows checked; no exact original DOI/title match. Missing metadata and version questions require human decision; NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F187" s="0" t="inlineStr">
@@ -25508,7 +25545,7 @@
       </c>
       <c r="N187" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T15:34:47Z</t>
+          <t xml:space="preserve">2026-10-30T02:33:23Z</t>
         </is>
       </c>
     </row>
@@ -25530,12 +25567,13 @@
       </c>
       <c r="D188" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="E188" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Version 1 of ELDORA ML QC dataset; article confirms WPO award and dataset link, native Figshare first publication date unresolved. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET: Version 1 of ELDORA ML QC dataset; article confirms WPO award and dataset link, native Figshare first publication date unresolved. Original DOI evaluated independently from expanded articles; complete 1238-row REACH index and all 53 existing Scout candidate rows checked; private reviewer decisions not accessible.
+REACH-SCOUT-2026-10-29-HOURLY-2229ET: One substantive bounded different-source recovery round; AMS article explicitly links exact dataset and WPO award; NOAA IR corroborates; Figshare API inaccessible; concept/v1 are same output family. Full REACH index 10/10 and detail 140/140 shards, SPARK 6/6 index, and Scout 17 immutable batches/59 rows checked; no exact original DOI/title match. Missing metadata and version questions require human decision; NOT DELIVERED TO HUB.</t>
         </is>
       </c>
       <c r="F188" s="0" t="inlineStr">
@@ -25580,7 +25618,7 @@
       </c>
       <c r="N188" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29T15:34:47Z</t>
+          <t xml:space="preserve">2026-10-30T02:33:23Z</t>
         </is>
       </c>
     </row>
@@ -26096,22 +26134,22 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://doi.org/10.6084/m9.figshare.23666259</t>
+          <t xml:space="preserve">https://doi.org/10.5281/zenodo.23044469</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://doi.org/10.1175/mwr-d-23-0144.1</t>
+          <t xml:space="preserve">https://doi.org/10.1029/2024wr037507</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Investigating Temporal Characteristics of Polarimetric and Electrical Signatures in Three Severe Storms: Insights from the VORTEX-Southeast Field Campaign</t>
+          <t xml:space="preserve">Assessing the Potential for Medium-Range Ice Forecasts in the Laurentian Great Lakes</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">NA19OAR4590209</t>
+          <t xml:space="preserve">NA22OAR4590188</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -26131,74 +26169,230 @@
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://repository.library.noaa.gov/view/noaa/70846</t>
+          <t xml:space="preserve">https://repository.library.noaa.gov/view/noaa/67984</t>
         </is>
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://github.com/PART-WPO/reach-scout-discoveries/blob/main/scout-discoveries/batches/2026-10-29-hourly-1131ET-verified-article-expansion-001.csv</t>
+          <t xml:space="preserve">https://github.com/PART-WPO/reach-scout-discoveries/blob/main/scout-discoveries/batches/2026-10-29-hourly-1929ET-verified-article-expansion-001.csv</t>
         </is>
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET</t>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1929ET</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">https://doi.org/10.5281/zenodo.23289230</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.1029/2024ms004319</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detecting Instantaneous Tidal Signals in Ocean Models Utilizing Streaming Band-Pass Filters</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA22OAR0110487</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API-seeded expansion</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Staged for human review; decision not verified</t>
+        </is>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://repository.library.noaa.gov/view/noaa/66967</t>
+        </is>
+      </c>
+      <c r="I10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://github.com/PART-WPO/reach-scout-discoveries/blob/main/scout-discoveries/batches/2026-10-29-hourly-1929ET-verified-article-expansion-001.csv</t>
+        </is>
+      </c>
+      <c r="J10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1929ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.5281/zenodo.23289230</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.1029/2025ms005126</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parameterization of Frequency-Dependent Internal Wave Drag in Global Ocean Models</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA22OAR0110487</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API-seeded expansion</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Staged for human review; decision not verified</t>
+        </is>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://repository.library.noaa.gov/view/noaa/73117</t>
+        </is>
+      </c>
+      <c r="I11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://github.com/PART-WPO/reach-scout-discoveries/blob/main/scout-discoveries/batches/2026-10-29-hourly-1929ET-verified-article-expansion-001.csv</t>
+        </is>
+      </c>
+      <c r="J11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1929ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.6084/m9.figshare.23666259</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.1175/mwr-d-23-0144.1</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Investigating Temporal Characteristics of Polarimetric and Electrical Signatures in Three Severe Storms: Insights from the VORTEX-Southeast Field Campaign</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA19OAR4590209</t>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API-seeded expansion</t>
+        </is>
+      </c>
+      <c r="F12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Staged for human review; decision not verified</t>
+        </is>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://repository.library.noaa.gov/view/noaa/70846</t>
+        </is>
+      </c>
+      <c r="I12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://github.com/PART-WPO/reach-scout-discoveries/blob/main/scout-discoveries/batches/2026-10-29-hourly-1131ET-verified-article-expansion-001.csv</t>
+        </is>
+      </c>
+      <c r="J12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://doi.org/10.6084/m9.figshare.23689194</t>
         </is>
       </c>
-      <c r="B10" s="0" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">https://doi.org/10.1175/aies-d-23-0064.1</t>
         </is>
       </c>
-      <c r="C10" s="0" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Airborne Radar Quality Control with Machine Learning</t>
         </is>
       </c>
-      <c r="D10" s="0" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">NA19OAR4590245</t>
         </is>
       </c>
-      <c r="E10" s="0" t="inlineStr">
+      <c r="E13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">API-seeded expansion</t>
         </is>
       </c>
-      <c r="F10" s="0" t="inlineStr">
+      <c r="F13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Staged for human review; decision not verified</t>
         </is>
       </c>
-      <c r="G10" s="0" t="inlineStr">
+      <c r="G13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">High</t>
         </is>
       </c>
-      <c r="H10" s="0" t="inlineStr">
+      <c r="H13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">https://repository.library.noaa.gov/view/noaa/64095</t>
         </is>
       </c>
-      <c r="I10" s="0" t="inlineStr">
+      <c r="I13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">https://github.com/PART-WPO/reach-scout-discoveries/blob/main/scout-discoveries/batches/2026-10-29-hourly-1131ET-verified-article-expansion-001.csv</t>
         </is>
       </c>
-      <c r="J10" s="0" t="inlineStr">
+      <c r="J13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">REACH-SCOUT-2026-10-29-HOURLY-1131ET</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J10"/>
+  <autoFilter ref="A1:J13"/>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -26668,10 +26862,10 @@
         <v>0</v>
       </c>
       <c r="F13" s="2">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G13" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
@@ -27053,10 +27247,10 @@
         <v>0</v>
       </c>
       <c r="F24" s="2">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G24" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H24" s="0" t="inlineStr">
         <is>
@@ -27712,7 +27906,7 @@
         <v>0</v>
       </c>
       <c r="D43" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E43" s="2">
         <v>0</v>
@@ -27721,7 +27915,7 @@
         <v>0</v>
       </c>
       <c r="G43" s="2">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H43" s="0" t="inlineStr">
         <is>
@@ -28523,10 +28717,10 @@
         <v>0</v>
       </c>
       <c r="F66" s="2">
+        <v>1</v>
+      </c>
+      <c r="G66" s="2">
         <v>0</v>
-      </c>
-      <c r="G66" s="2">
-        <v>1</v>
       </c>
       <c r="H66" s="0" t="inlineStr">
         <is>
@@ -28612,7 +28806,7 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C2" s="0" t="inlineStr">
         <is>
@@ -28623,30 +28817,30 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Further research scheduled; not cleared</t>
+          <t xml:space="preserve">Already represented in REACH</t>
         </is>
       </c>
       <c r="B3" s="2">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Possible output, but required dates, eligibility, unique identity or project attribution are unresolved.</t>
+          <t xml:space="preserve">Scout located the output or its version-family in REACH; no duplicate addition is implied.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Already represented in REACH</t>
+          <t xml:space="preserve">Human metadata assistance needed; not approved</t>
         </is>
       </c>
       <c r="B4" s="2">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scout located the output or its version-family in REACH; no duplicate addition is implied.</t>
+          <t xml:space="preserve">Evidence suggests a relevant output but missing required details need human help.</t>
         </is>
       </c>
     </row>
@@ -28672,7 +28866,7 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>

</xml_diff>